<commit_message>
v10.17: Further Playwright Configuration
</commit_message>
<xml_diff>
--- a/PMS/tests/test-assets/user-list/invalid_data.xlsx
+++ b/PMS/tests/test-assets/user-list/invalid_data.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="10">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -50,12 +50,6 @@
   </si>
   <si>
     <t xml:space="preserve">supervisor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ingest3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ingest3@uni.com</t>
   </si>
 </sst>
 </file>
@@ -70,6 +64,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -129,8 +124,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -261,60 +260,52 @@
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="0" t="n">
+      <c r="B3" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="0" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="0" t="s">
-        <v>6</v>
-      </c>
-      <c r="D4" s="0" t="n">
-        <v>1</v>
-      </c>
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>